<commit_message>
Added imgs for DT explanation
</commit_message>
<xml_diff>
--- a/Machine_Learning/Dataset/ML_data1.xlsx
+++ b/Machine_Learning/Dataset/ML_data1.xlsx
@@ -1,13 +1,22 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30430"/>
   <workbookPr/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ELCOT\Desktop\JananiMurugan\Machine_Learning\Dataset\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ED22ACAB-8C1B-426F-BB0A-CD3634C4BFEC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <bookViews>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+  </bookViews>
   <sheets>
-    <sheet state="visible" name="Sheet1" sheetId="1" r:id="rId5"/>
-    <sheet state="visible" name="Sheet2" sheetId="2" r:id="rId6"/>
+    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="Model_Dev" sheetId="2" r:id="rId2"/>
   </sheets>
-  <definedNames/>
-  <calcPr/>
+  <calcPr calcId="0"/>
 </workbook>
 </file>
 
@@ -98,21 +107,23 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-  <fonts count="3">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
-      <sz val="10.0"/>
+      <sz val="10"/>
       <color rgb="FF000000"/>
       <name val="Arial"/>
       <scheme val="minor"/>
     </font>
     <font>
       <b/>
+      <sz val="10"/>
       <color theme="1"/>
       <name val="Arial"/>
       <scheme val="minor"/>
     </font>
     <font>
+      <sz val="10"/>
       <color theme="1"/>
       <name val="Arial"/>
       <scheme val="minor"/>
@@ -123,7 +134,7 @@
       <patternFill patternType="none"/>
     </fill>
     <fill>
-      <patternFill patternType="lightGray"/>
+      <patternFill patternType="gray125"/>
     </fill>
     <fill>
       <patternFill patternType="solid">
@@ -133,7 +144,13 @@
     </fill>
   </fills>
   <borders count="2">
-    <border/>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
     <border>
       <left style="thin">
         <color rgb="FF000000"/>
@@ -147,58 +164,50 @@
       <bottom style="thin">
         <color rgb="FF000000"/>
       </bottom>
+      <diagonal/>
     </border>
   </borders>
   <cellStyleXfs count="1">
-    <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
   <cellXfs count="8">
-    <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
     </xf>
-    <xf borderId="1" fillId="2" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
-      <alignment horizontal="right" readingOrder="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
-    <xf borderId="1" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment horizontal="center" readingOrder="0"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
-    <xf borderId="1" fillId="2" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
-      <alignment horizontal="center" readingOrder="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
     </xf>
-    <xf borderId="1" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment horizontal="right" readingOrder="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
     </xf>
-    <xf borderId="1" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment horizontal="right" readingOrder="0"/>
-    </xf>
-    <xf borderId="1" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment readingOrder="0"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment readingOrder="0"/>
-    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle xfId="0" name="Normal" builtinId="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
+  <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
+  </extLst>
 </styleSheet>
 </file>
 
-<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
-<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:cx="http://schemas.microsoft.com/office/drawing/2014/chartex" xmlns:cx1="http://schemas.microsoft.com/office/drawing/2015/9/8/chartex" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:dgm="http://schemas.openxmlformats.org/drawingml/2006/diagram" xmlns:x3Unk="http://schemas.microsoft.com/office/drawing/2010/slicer" xmlns:sle15="http://schemas.microsoft.com/office/drawing/2012/slicer"/>
-</file>
-
-<file path=xl/drawings/drawing2.xml><?xml version="1.0" encoding="utf-8"?>
-<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:cx="http://schemas.microsoft.com/office/drawing/2014/chartex" xmlns:cx1="http://schemas.microsoft.com/office/drawing/2015/9/8/chartex" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:dgm="http://schemas.openxmlformats.org/drawingml/2006/diagram" xmlns:x3Unk="http://schemas.microsoft.com/office/drawing/2010/slicer" xmlns:sle15="http://schemas.microsoft.com/office/drawing/2012/slicer"/>
-</file>
-
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<x18tc:personList xmlns:x18tc="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments"/>
-</file>
-
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheets">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Sheets">
   <a:themeElements>
     <a:clrScheme name="Sheets">
       <a:dk1>
@@ -388,17 +397,20 @@
       </a:bgFillStyleLst>
     </a:fmtScheme>
   </a:themeElements>
+  <a:objectDefaults/>
+  <a:extraClrSchemeLst/>
 </a:theme>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
-  <sheetFormatPr customHeight="1" defaultColWidth="12.63" defaultRowHeight="15.75"/>
+  <dimension ref="A1:H13"/>
+  <sheetFormatPr defaultColWidth="12.5703125" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
   <sheetData>
-    <row r="1">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -424,24 +436,24 @@
         <v>7</v>
       </c>
     </row>
-    <row r="2">
+    <row r="2" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A2" s="5">
-        <v>101.0</v>
+        <v>101</v>
       </c>
       <c r="B2" s="6" t="s">
         <v>14</v>
       </c>
       <c r="C2" s="5">
-        <v>85.0</v>
+        <v>85</v>
       </c>
       <c r="D2" s="5">
-        <v>78.0</v>
+        <v>78</v>
       </c>
       <c r="E2" s="5">
-        <v>12.0</v>
+        <v>12</v>
       </c>
       <c r="F2" s="5">
-        <v>0.0</v>
+        <v>0</v>
       </c>
       <c r="G2" s="6" t="s">
         <v>15</v>
@@ -450,24 +462,24 @@
         <v>16</v>
       </c>
     </row>
-    <row r="3">
+    <row r="3" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A3" s="5">
-        <v>102.0</v>
+        <v>102</v>
       </c>
       <c r="B3" s="6" t="s">
         <v>17</v>
       </c>
       <c r="C3" s="5">
-        <v>62.0</v>
+        <v>62</v>
       </c>
       <c r="D3" s="5">
-        <v>45.0</v>
+        <v>45</v>
       </c>
       <c r="E3" s="5">
-        <v>5.0</v>
+        <v>5</v>
       </c>
       <c r="F3" s="5">
-        <v>2.0</v>
+        <v>2</v>
       </c>
       <c r="G3" s="6" t="s">
         <v>18</v>
@@ -476,24 +488,24 @@
         <v>19</v>
       </c>
     </row>
-    <row r="4">
+    <row r="4" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A4" s="5">
-        <v>103.0</v>
+        <v>103</v>
       </c>
       <c r="B4" s="6" t="s">
         <v>14</v>
       </c>
       <c r="C4" s="5">
-        <v>91.0</v>
+        <v>91</v>
       </c>
       <c r="D4" s="5">
-        <v>88.0</v>
+        <v>88</v>
       </c>
       <c r="E4" s="5">
-        <v>15.0</v>
+        <v>15</v>
       </c>
       <c r="F4" s="5">
-        <v>0.0</v>
+        <v>0</v>
       </c>
       <c r="G4" s="6" t="s">
         <v>15</v>
@@ -502,24 +514,24 @@
         <v>16</v>
       </c>
     </row>
-    <row r="5">
+    <row r="5" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A5" s="5">
-        <v>104.0</v>
+        <v>104</v>
       </c>
       <c r="B5" s="6" t="s">
         <v>20</v>
       </c>
       <c r="C5" s="5">
-        <v>74.0</v>
+        <v>74</v>
       </c>
       <c r="D5" s="5" t="s">
         <v>21</v>
       </c>
       <c r="E5" s="5">
-        <v>8.0</v>
+        <v>8</v>
       </c>
       <c r="F5" s="5">
-        <v>1.0</v>
+        <v>1</v>
       </c>
       <c r="G5" s="6" t="s">
         <v>18</v>
@@ -528,24 +540,24 @@
         <v>16</v>
       </c>
     </row>
-    <row r="6">
+    <row r="6" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A6" s="5">
-        <v>105.0</v>
+        <v>105</v>
       </c>
       <c r="B6" s="6" t="s">
         <v>17</v>
       </c>
       <c r="C6" s="5">
-        <v>55.0</v>
+        <v>55</v>
       </c>
       <c r="D6" s="5">
-        <v>39.0</v>
+        <v>39</v>
       </c>
       <c r="E6" s="5">
-        <v>4.0</v>
+        <v>4</v>
       </c>
       <c r="F6" s="5">
-        <v>3.0</v>
+        <v>3</v>
       </c>
       <c r="G6" s="6" t="s">
         <v>15</v>
@@ -554,7 +566,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="11">
+    <row r="11" spans="1:8" x14ac:dyDescent="0.2">
       <c r="D11" s="7" t="s">
         <v>22</v>
       </c>
@@ -565,41 +577,55 @@
         <v>24</v>
       </c>
     </row>
-    <row r="12">
+    <row r="12" spans="1:8" x14ac:dyDescent="0.2">
       <c r="D12" s="7">
-        <v>90.0</v>
+        <v>90</v>
       </c>
       <c r="E12" s="7">
-        <v>76.0</v>
+        <v>76</v>
       </c>
       <c r="F12" s="7">
-        <v>56.0</v>
-      </c>
-    </row>
-    <row r="13">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="13" spans="1:8" x14ac:dyDescent="0.2">
       <c r="D13" s="7">
-        <v>90.0</v>
+        <v>90</v>
       </c>
       <c r="E13" s="7">
-        <v>89.0</v>
+        <v>89</v>
       </c>
       <c r="F13" s="7">
-        <v>78.0</v>
+        <v>78</v>
       </c>
     </row>
   </sheetData>
-  <drawing r:id="rId1"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
-  <sheetFormatPr customHeight="1" defaultColWidth="12.63" defaultRowHeight="15.75"/>
+  <dimension ref="A1:K6"/>
+  <sheetFormatPr defaultColWidth="12.5703125" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="1" max="1" width="10.85546875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="11.5703125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="11.28515625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="12.28515625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="18" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="14.42578125" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="14" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="9.140625" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="13.7109375" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="11.85546875" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="9.5703125" bestFit="1" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1">
+    <row r="1" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
@@ -634,182 +660,182 @@
         <v>13</v>
       </c>
     </row>
-    <row r="2">
+    <row r="2" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A2" s="6">
-        <v>1001.0</v>
+        <v>1001</v>
       </c>
       <c r="B2" s="6" t="s">
         <v>14</v>
       </c>
       <c r="C2" s="5">
-        <v>92.0</v>
+        <v>92</v>
       </c>
       <c r="D2" s="5">
-        <v>8.0</v>
+        <v>8</v>
       </c>
       <c r="E2" s="5">
-        <v>88.0</v>
+        <v>88</v>
       </c>
       <c r="F2" s="5">
-        <v>82.0</v>
+        <v>82</v>
       </c>
       <c r="G2" s="5">
         <v>8.6</v>
       </c>
       <c r="H2" s="5">
-        <v>0.0</v>
+        <v>0</v>
       </c>
       <c r="I2" s="5">
-        <v>6.0</v>
+        <v>6</v>
       </c>
       <c r="J2" s="5">
-        <v>87.0</v>
+        <v>87</v>
       </c>
       <c r="K2" s="6" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="3">
+    <row r="3" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A3" s="6">
-        <v>1002.0</v>
+        <v>1002</v>
       </c>
       <c r="B3" s="6" t="s">
         <v>17</v>
       </c>
       <c r="C3" s="5">
-        <v>76.0</v>
+        <v>76</v>
       </c>
       <c r="D3" s="5">
-        <v>5.0</v>
+        <v>5</v>
       </c>
       <c r="E3" s="5">
-        <v>72.0</v>
+        <v>72</v>
       </c>
       <c r="F3" s="5">
-        <v>68.0</v>
+        <v>68</v>
       </c>
       <c r="G3" s="5">
         <v>7.2</v>
       </c>
       <c r="H3" s="5">
-        <v>1.0</v>
+        <v>1</v>
       </c>
       <c r="I3" s="5">
-        <v>3.0</v>
+        <v>3</v>
       </c>
       <c r="J3" s="5">
-        <v>71.0</v>
+        <v>71</v>
       </c>
       <c r="K3" s="6" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="4">
+    <row r="4" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A4" s="6">
-        <v>1003.0</v>
+        <v>1003</v>
       </c>
       <c r="B4" s="6" t="s">
         <v>20</v>
       </c>
       <c r="C4" s="5">
-        <v>61.0</v>
+        <v>61</v>
       </c>
       <c r="D4" s="5">
         <v>3.5</v>
       </c>
       <c r="E4" s="5">
-        <v>55.0</v>
+        <v>55</v>
       </c>
       <c r="F4" s="5">
-        <v>52.0</v>
+        <v>52</v>
       </c>
       <c r="G4" s="5">
         <v>6.4</v>
       </c>
       <c r="H4" s="5">
-        <v>3.0</v>
+        <v>3</v>
       </c>
       <c r="I4" s="5">
-        <v>1.0</v>
+        <v>1</v>
       </c>
       <c r="J4" s="5">
-        <v>54.0</v>
+        <v>54</v>
       </c>
       <c r="K4" s="6" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="5">
+    <row r="5" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A5" s="6">
-        <v>1004.0</v>
+        <v>1004</v>
       </c>
       <c r="B5" s="6" t="s">
         <v>25</v>
       </c>
       <c r="C5" s="5">
-        <v>95.0</v>
+        <v>95</v>
       </c>
       <c r="D5" s="5">
-        <v>9.0</v>
+        <v>9</v>
       </c>
       <c r="E5" s="5">
-        <v>94.0</v>
+        <v>94</v>
       </c>
       <c r="F5" s="5">
-        <v>91.0</v>
+        <v>91</v>
       </c>
       <c r="G5" s="5">
         <v>9.1</v>
       </c>
       <c r="H5" s="5">
-        <v>0.0</v>
+        <v>0</v>
       </c>
       <c r="I5" s="5">
-        <v>8.0</v>
+        <v>8</v>
       </c>
       <c r="J5" s="5">
-        <v>93.0</v>
+        <v>93</v>
       </c>
       <c r="K5" s="6" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="6">
+    <row r="6" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A6" s="6">
-        <v>1005.0</v>
+        <v>1005</v>
       </c>
       <c r="B6" s="6" t="s">
         <v>26</v>
       </c>
       <c r="C6" s="5">
-        <v>68.0</v>
+        <v>68</v>
       </c>
       <c r="D6" s="5">
-        <v>4.0</v>
+        <v>4</v>
       </c>
       <c r="E6" s="5">
-        <v>61.0</v>
+        <v>61</v>
       </c>
       <c r="F6" s="5">
-        <v>58.0</v>
+        <v>58</v>
       </c>
       <c r="G6" s="5">
         <v>6.8</v>
       </c>
       <c r="H6" s="5">
-        <v>2.0</v>
+        <v>2</v>
       </c>
       <c r="I6" s="5">
-        <v>2.0</v>
+        <v>2</v>
       </c>
       <c r="J6" s="5">
-        <v>60.0</v>
+        <v>60</v>
       </c>
       <c r="K6" s="6" t="s">
         <v>16</v>
       </c>
     </row>
   </sheetData>
-  <drawing r:id="rId1"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>